<commit_message>
Complete Material to Building pipeline & Database
- Missing WindowMaterial implementation
- README.md is not up to date
</commit_message>
<xml_diff>
--- a/Material_Database.xlsx
+++ b/Material_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djami\Documents\GitHub\EPSM_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE3824A-4E19-46E0-83CD-09569964381F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28622119-AE87-4B47-9140-0EDB1444FB6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="4" xr2:uid="{674BB936-5EA3-D94C-A89F-A01CB7CEE187}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{674BB936-5EA3-D94C-A89F-A01CB7CEE187}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Notes" sheetId="5" r:id="rId1"/>
@@ -52,15 +52,17 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={3206CACE-8394-4121-9269-0EA8CAAF86B2}</author>
+    <author>tc={180FB3EA-0C67-43EA-8C29-284FB4E1924C}</author>
     <author>tc={2113958F-D93A-4B72-9A27-4CE4FBEEAA3B}</author>
     <author>tc={E3B66A5C-4257-4423-90E2-3C4F485F94E4}</author>
     <author>tc={63E75155-291D-404C-B313-1AF4E66194E8}</author>
     <author>tc={B2A9821F-0147-4752-848D-F3C9C655B99C}</author>
     <author>tc={BB4FC2B9-BA1F-4EA5-B691-CF3EA295DA25}</author>
     <author>tc={261C8EBC-4D03-4C47-A332-27A70C92E6E5}</author>
+    <author>tc={A6D8CDDA-498D-4A56-87AC-DDCDC6FBE328}</author>
     <author>tc={19159A99-372E-4AEB-A2A3-8A2620179DC6}</author>
     <author>tc={4768D1CA-0281-489C-8890-493EDF2E42FC}</author>
+    <author>tc={F8C9E8B1-B583-4393-9FBA-92446F147450}</author>
     <author>tc={6B629ABE-2EFA-4F2C-AD59-8B48A4573FA8}</author>
     <author>tc={D1C85F94-74D2-4C40-B2A6-CAE72652D12D}</author>
     <author>tc={31404CAB-DC9F-4DFA-BB4E-FBD9ADD6D463}</author>
@@ -83,12 +85,12 @@
     <author>tc={1FEFA72F-4293-4A15-AC93-B61BCFC6CC2A}</author>
   </authors>
   <commentList>
-    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{3206CACE-8394-4121-9269-0EA8CAAF86B2}">
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{180FB3EA-0C67-43EA-8C29-284FB4E1924C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Generic metal surface</t>
+    https://www.metalsupermarkets.co.uk/product/mild-steel-sheet-galvanised/#:~:text=Framework,Thermal%20Expansion:%2012.06%20%C2%B5m/m%2Dk</t>
       </text>
     </comment>
     <comment ref="A8" authorId="1" shapeId="0" xr:uid="{2113958F-D93A-4B72-9A27-4CE4FBEEAA3B}">
@@ -112,9 +114,7 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Specific heat matched closest w value given in https://www.mdpi.com/2673-4109/2/1/14 
-alt. M11 100mm lightweight concrete 
-Density in SS-EN ISO 10456  for Concrete with more than 70 % expanded blast-furnace slag aggregate is 1100-1700 (Dry sand from json is about 1500)</t>
+    SS-EN ISO 10456, Table 4</t>
       </text>
     </comment>
     <comment ref="E10" authorId="4" shapeId="0" xr:uid="{B2A9821F-0147-4752-848D-F3C9C655B99C}">
@@ -122,16 +122,15 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    25mm Stucco
-Fits better according to ISO</t>
+    Table 3</t>
       </text>
     </comment>
     <comment ref="E11" authorId="5" shapeId="0" xr:uid="{BB4FC2B9-BA1F-4EA5-B691-CF3EA295DA25}">
       <text>
-        <t>[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Works with autoclaved concrete given in SS-EN ISO 10456 (based on density and specific heat capacity)</t>
+    autoclaved concrete Table 4, SS-EN ISO 10456 </t>
       </text>
     </comment>
     <comment ref="C12" authorId="6" shapeId="0" xr:uid="{261C8EBC-4D03-4C47-A332-27A70C92E6E5}">
@@ -142,7 +141,15 @@
     Terrasit is a specific brand of plaster that utilises EPS (Expanding Polystyrene)</t>
       </text>
     </comment>
-    <comment ref="A15" authorId="7" shapeId="0" xr:uid="{19159A99-372E-4AEB-A2A3-8A2620179DC6}">
+    <comment ref="E12" authorId="7" shapeId="0" xr:uid="{A6D8CDDA-498D-4A56-87AC-DDCDC6FBE328}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Conductivity might be low compared to others (cement, sand: Table 3)</t>
+      </text>
+    </comment>
+    <comment ref="A15" authorId="8" shapeId="0" xr:uid="{19159A99-372E-4AEB-A2A3-8A2620179DC6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -150,7 +157,7 @@
     identical to plaster</t>
       </text>
     </comment>
-    <comment ref="C16" authorId="8" shapeId="0" xr:uid="{4768D1CA-0281-489C-8890-493EDF2E42FC}">
+    <comment ref="C16" authorId="9" shapeId="0" xr:uid="{4768D1CA-0281-489C-8890-493EDF2E42FC}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -158,7 +165,15 @@
      desc: Wood wool panels are made by mixing wood shavings with cement and lime as a binder and any paint.</t>
       </text>
     </comment>
-    <comment ref="E17" authorId="9" shapeId="0" xr:uid="{6B629ABE-2EFA-4F2C-AD59-8B48A4573FA8}">
+    <comment ref="E16" authorId="10" shapeId="0" xr:uid="{F8C9E8B1-B583-4393-9FBA-92446F147450}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Cement bonded particle board, Table 3</t>
+      </text>
+    </comment>
+    <comment ref="E17" authorId="11" shapeId="0" xr:uid="{6B629ABE-2EFA-4F2C-AD59-8B48A4573FA8}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -167,7 +182,7 @@
 https://www.engineeringtoolbox.com/thermal-conductivity-d_429.html</t>
       </text>
     </comment>
-    <comment ref="C18" authorId="10" shapeId="0" xr:uid="{D1C85F94-74D2-4C40-B2A6-CAE72652D12D}">
+    <comment ref="C18" authorId="12" shapeId="0" xr:uid="{D1C85F94-74D2-4C40-B2A6-CAE72652D12D}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -175,7 +190,7 @@
     metal is a bit arbitrary</t>
       </text>
     </comment>
-    <comment ref="C21" authorId="11" shapeId="0" xr:uid="{31404CAB-DC9F-4DFA-BB4E-FBD9ADD6D463}">
+    <comment ref="C21" authorId="13" shapeId="0" xr:uid="{31404CAB-DC9F-4DFA-BB4E-FBD9ADD6D463}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -183,7 +198,7 @@
     closest</t>
       </text>
     </comment>
-    <comment ref="C24" authorId="12" shapeId="0" xr:uid="{AC4C6092-4E4D-460F-BFF6-05E9D096651F}">
+    <comment ref="C24" authorId="14" shapeId="0" xr:uid="{AC4C6092-4E4D-460F-BFF6-05E9D096651F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -191,7 +206,7 @@
     stenull</t>
       </text>
     </comment>
-    <comment ref="E24" authorId="13" shapeId="0" xr:uid="{C76F23C2-744A-4F5B-8E93-C92988DCEE50}">
+    <comment ref="E24" authorId="15" shapeId="0" xr:uid="{C76F23C2-744A-4F5B-8E93-C92988DCEE50}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -199,7 +214,7 @@
     Based on closest conductivity match</t>
       </text>
     </comment>
-    <comment ref="C27" authorId="14" shapeId="0" xr:uid="{E593AE45-BFBC-4A98-85EB-1F88F0EF546C}">
+    <comment ref="C27" authorId="16" shapeId="0" xr:uid="{E593AE45-BFBC-4A98-85EB-1F88F0EF546C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -207,7 +222,7 @@
     similar but without the asbestos</t>
       </text>
     </comment>
-    <comment ref="E27" authorId="15" shapeId="0" xr:uid="{718A134D-676E-4A8A-B271-F30AAE35BC96}">
+    <comment ref="E27" authorId="17" shapeId="0" xr:uid="{718A134D-676E-4A8A-B271-F30AAE35BC96}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -215,7 +230,7 @@
     https://help.iesve.com/ve2021/table_6_thermal_conductivity__specific_heat_capacity_and_density.htm</t>
       </text>
     </comment>
-    <comment ref="C28" authorId="16" shapeId="0" xr:uid="{F356163D-CC1D-44C8-933A-745241019FA2}">
+    <comment ref="C28" authorId="18" shapeId="0" xr:uid="{F356163D-CC1D-44C8-933A-745241019FA2}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -223,7 +238,7 @@
     Contains bitumen, otherwise 6000000140</t>
       </text>
     </comment>
-    <comment ref="E28" authorId="17" shapeId="0" xr:uid="{87C1EFB4-FED1-400C-B715-2FFCC96D5F2D}">
+    <comment ref="E28" authorId="19" shapeId="0" xr:uid="{87C1EFB4-FED1-400C-B715-2FFCC96D5F2D}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -231,7 +246,7 @@
     https://help.iesve.com/ve2021/table_6_thermal_conductivity__specific_heat_capacity_and_density.htm</t>
       </text>
     </comment>
-    <comment ref="C29" authorId="18" shapeId="0" xr:uid="{E60A6551-649A-4C04-95E1-FA84B1B69D7E}">
+    <comment ref="C29" authorId="20" shapeId="0" xr:uid="{E60A6551-649A-4C04-95E1-FA84B1B69D7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -239,7 +254,7 @@
     Closest plastic product</t>
       </text>
     </comment>
-    <comment ref="C31" authorId="19" shapeId="0" xr:uid="{7268449F-3191-428A-8371-DD50056F1F43}">
+    <comment ref="C31" authorId="21" shapeId="0" xr:uid="{7268449F-3191-428A-8371-DD50056F1F43}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -247,7 +262,7 @@
     lättklinkerkulor</t>
       </text>
     </comment>
-    <comment ref="E32" authorId="20" shapeId="0" xr:uid="{3F43729D-EBB4-4593-A275-FE8B53D78FEA}">
+    <comment ref="E32" authorId="22" shapeId="0" xr:uid="{3F43729D-EBB4-4593-A275-FE8B53D78FEA}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -255,7 +270,7 @@
     Based on closest conductivity match</t>
       </text>
     </comment>
-    <comment ref="E33" authorId="21" shapeId="0" xr:uid="{E7C52893-AA17-450F-920D-11C21788EBD9}">
+    <comment ref="E33" authorId="23" shapeId="0" xr:uid="{E7C52893-AA17-450F-920D-11C21788EBD9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -263,7 +278,7 @@
     Based on closest conductivity match</t>
       </text>
     </comment>
-    <comment ref="E36" authorId="22" shapeId="0" xr:uid="{23F12E34-1B4E-45BB-A08F-8B64E51E0389}">
+    <comment ref="E36" authorId="24" shapeId="0" xr:uid="{23F12E34-1B4E-45BB-A08F-8B64E51E0389}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -271,7 +286,7 @@
     https://help.iesve.com/ve2021/table_6_thermal_conductivity__specific_heat_capacity_and_density.htm</t>
       </text>
     </comment>
-    <comment ref="C40" authorId="23" shapeId="0" xr:uid="{18D9EEC2-9764-4F05-BDEE-1F7F69B611F4}">
+    <comment ref="C40" authorId="25" shapeId="0" xr:uid="{18D9EEC2-9764-4F05-BDEE-1F7F69B611F4}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -279,7 +294,7 @@
     either or for lightweight</t>
       </text>
     </comment>
-    <comment ref="E43" authorId="24" shapeId="0" xr:uid="{C91F94D8-8AD2-4074-803D-F77C2526C8D2}">
+    <comment ref="E43" authorId="26" shapeId="0" xr:uid="{C91F94D8-8AD2-4074-803D-F77C2526C8D2}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -287,7 +302,7 @@
     https://materialsark.com/faqs/thermal-conductivity/</t>
       </text>
     </comment>
-    <comment ref="E45" authorId="25" shapeId="0" xr:uid="{16296FEB-3037-4598-AEB7-E2D43462D860}">
+    <comment ref="E45" authorId="27" shapeId="0" xr:uid="{16296FEB-3037-4598-AEB7-E2D43462D860}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -295,7 +310,7 @@
     Least dense wood material</t>
       </text>
     </comment>
-    <comment ref="C47" authorId="26" shapeId="0" xr:uid="{FEF83151-61B5-496E-9EF9-E10E1AF7F09C}">
+    <comment ref="C47" authorId="28" shapeId="0" xr:uid="{FEF83151-61B5-496E-9EF9-E10E1AF7F09C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -303,7 +318,7 @@
     Plastic product used as a vapor barrier, if thickness is accounted for perhaps it’s the closest</t>
       </text>
     </comment>
-    <comment ref="A54" authorId="27" shapeId="0" xr:uid="{F2014166-D5BD-416D-A5A9-D7840AFC5CE3}">
+    <comment ref="A54" authorId="29" shapeId="0" xr:uid="{F2014166-D5BD-416D-A5A9-D7840AFC5CE3}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -313,7 +328,7 @@
     Copied from metal_sheet</t>
       </text>
     </comment>
-    <comment ref="C54" authorId="28" shapeId="0" xr:uid="{1FEFA72F-4293-4A15-AC93-B61BCFC6CC2A}">
+    <comment ref="C54" authorId="30" shapeId="0" xr:uid="{1FEFA72F-4293-4A15-AC93-B61BCFC6CC2A}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -398,7 +413,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1592" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1592" uniqueCount="540">
   <si>
     <t>Date</t>
   </si>
@@ -2052,6 +2067,12 @@
   <si>
     <t>Wood Frame NonRes Wall Insulation-0.73</t>
   </si>
+  <si>
+    <t>25mm Stucco</t>
+  </si>
+  <si>
+    <t>NACM_Gypsum Board 5/8in</t>
+  </si>
 </sst>
 </file>
 
@@ -2060,7 +2081,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="29" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2237,6 +2258,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="21">
@@ -2595,7 +2622,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="169">
+  <cellXfs count="171">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2840,7 +2867,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2848,6 +2874,13 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3792,8 +3825,14 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="E7" dT="2026-02-11T13:27:32.61" personId="{B922D462-EEF4-49CB-AA8E-A16643E336EE}" id="{3206CACE-8394-4121-9269-0EA8CAAF86B2}">
-    <text>Generic metal surface</text>
+  <threadedComment ref="E7" dT="2026-02-24T21:21:39.03" personId="{B922D462-EEF4-49CB-AA8E-A16643E336EE}" id="{180FB3EA-0C67-43EA-8C29-284FB4E1924C}">
+    <text>https://www.metalsupermarkets.co.uk/product/mild-steel-sheet-galvanised/#:~:text=Framework,Thermal%20Expansion:%2012.06%20%C2%B5m/m%2Dk</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>1339517197</xltc2:checksum>
+        <xltc2:hyperlink startIndex="0" length="135" url="https://www.metalsupermarkets.co.uk/product/mild-steel-sheet-galvanised/#:~:text=Framework,Thermal%20Expansion:%2012.06%20%C2%B5m/m%2Dk"/>
+      </x:ext>
+    </extLst>
   </threadedComment>
   <threadedComment ref="A8" dT="2026-01-21T15:19:25.37" personId="{B4433DAF-B1B3-3C42-9739-78512C18A3E2}" id="{2113958F-D93A-4B72-9A27-4CE4FBEEAA3B}">
     <text>boverket and json doesnt contain any gravel type materials</text>
@@ -3802,31 +3841,28 @@
     <text>Restproducts that are sometimes used are similar</text>
   </threadedComment>
   <threadedComment ref="E8" dT="2026-02-04T00:20:37.84" personId="{B922D462-EEF4-49CB-AA8E-A16643E336EE}" id="{63E75155-291D-404C-B313-1AF4E66194E8}">
-    <text>Specific heat matched closest w value given in https://www.mdpi.com/2673-4109/2/1/14 
-alt. M11 100mm lightweight concrete 
-Density in SS-EN ISO 10456  for Concrete with more than 70 % expanded blast-furnace slag aggregate is 1100-1700 (Dry sand from json is about 1500)</text>
-    <extLst>
-      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
-        <xltc2:checksum>2363598260</xltc2:checksum>
-        <xltc2:hyperlink startIndex="47" length="37" url="https://www.mdpi.com/2673-4109/2/1/14"/>
-      </x:ext>
-    </extLst>
+    <text>SS-EN ISO 10456, Table 4</text>
   </threadedComment>
   <threadedComment ref="E10" dT="2026-02-11T13:40:56.15" personId="{B922D462-EEF4-49CB-AA8E-A16643E336EE}" id="{B2A9821F-0147-4752-848D-F3C9C655B99C}">
-    <text>25mm Stucco
-Fits better according to ISO</text>
+    <text>Table 3</text>
   </threadedComment>
   <threadedComment ref="E11" dT="2026-02-11T13:55:59.21" personId="{B922D462-EEF4-49CB-AA8E-A16643E336EE}" id="{BB4FC2B9-BA1F-4EA5-B691-CF3EA295DA25}">
-    <text>Works with autoclaved concrete given in SS-EN ISO 10456 (based on density and specific heat capacity)</text>
+    <text xml:space="preserve">autoclaved concrete Table 4, SS-EN ISO 10456 </text>
   </threadedComment>
   <threadedComment ref="C12" dT="2026-02-04T18:34:50.50" personId="{B922D462-EEF4-49CB-AA8E-A16643E336EE}" id="{261C8EBC-4D03-4C47-A332-27A70C92E6E5}">
     <text>Terrasit is a specific brand of plaster that utilises EPS (Expanding Polystyrene)</text>
+  </threadedComment>
+  <threadedComment ref="E12" dT="2026-02-24T21:48:00.47" personId="{B922D462-EEF4-49CB-AA8E-A16643E336EE}" id="{A6D8CDDA-498D-4A56-87AC-DDCDC6FBE328}">
+    <text>Conductivity might be low compared to others (cement, sand: Table 3)</text>
   </threadedComment>
   <threadedComment ref="A15" dT="2025-12-05T07:06:02.23" personId="{B4433DAF-B1B3-3C42-9739-78512C18A3E2}" id="{19159A99-372E-4AEB-A2A3-8A2620179DC6}">
     <text>identical to plaster</text>
   </threadedComment>
   <threadedComment ref="C16" dT="2025-12-04T20:31:52.40" personId="{B4433DAF-B1B3-3C42-9739-78512C18A3E2}" id="{4768D1CA-0281-489C-8890-493EDF2E42FC}">
     <text> desc: Wood wool panels are made by mixing wood shavings with cement and lime as a binder and any paint.</text>
+  </threadedComment>
+  <threadedComment ref="E16" dT="2026-02-24T21:59:54.11" personId="{B922D462-EEF4-49CB-AA8E-A16643E336EE}" id="{F8C9E8B1-B583-4393-9FBA-92446F147450}">
+    <text>Cement bonded particle board, Table 3</text>
   </threadedComment>
   <threadedComment ref="E17" dT="2026-02-04T00:45:00.74" personId="{B922D462-EEF4-49CB-AA8E-A16643E336EE}" id="{6B629ABE-2EFA-4F2C-AD59-8B48A4573FA8}">
     <text>Closest when comparing values https://www.engineeringtoolbox.com/specific-heat-solids-d_154.html
@@ -16504,8 +16540,8 @@
       <c r="D7" s="37">
         <v>8</v>
       </c>
-      <c r="E7" s="140" t="s">
-        <v>72</v>
+      <c r="E7" s="36" t="s">
+        <v>108</v>
       </c>
       <c r="F7" s="36">
         <v>6</v>
@@ -16544,21 +16580,21 @@
         <v>73</v>
       </c>
       <c r="B8" s="36"/>
-      <c r="C8" s="137">
+      <c r="C8" s="145">
         <v>6000000085</v>
       </c>
-      <c r="D8" s="39">
+      <c r="D8" s="36">
         <v>3</v>
       </c>
-      <c r="E8" s="141" t="s">
-        <v>534</v>
+      <c r="E8" s="137" t="s">
+        <v>79</v>
       </c>
       <c r="F8" s="39">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G8" s="37">
         <f>(D8+F8)/2</f>
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="H8" s="14"/>
       <c r="I8" s="61"/>
@@ -16653,11 +16689,11 @@
         <v>75</v>
       </c>
       <c r="F9" s="36">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G9" s="37">
         <f t="shared" si="0"/>
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="I9" s="61"/>
       <c r="J9" s="61"/>
@@ -16696,7 +16732,7 @@
         <v>10</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>77</v>
+        <v>538</v>
       </c>
       <c r="F10" s="36">
         <v>10</v>
@@ -16742,7 +16778,7 @@
         <v>8</v>
       </c>
       <c r="E11" s="36" t="s">
-        <v>79</v>
+        <v>539</v>
       </c>
       <c r="F11" s="36">
         <v>10</v>
@@ -16788,7 +16824,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>77</v>
+        <v>538</v>
       </c>
       <c r="F12" s="36">
         <v>8</v>
@@ -16833,7 +16869,7 @@
       <c r="D13" s="37">
         <v>9</v>
       </c>
-      <c r="E13" s="36" t="s">
+      <c r="E13" s="37" t="s">
         <v>77</v>
       </c>
       <c r="F13" s="36">
@@ -16879,7 +16915,7 @@
       <c r="D14" s="40">
         <v>5</v>
       </c>
-      <c r="E14" s="137" t="s">
+      <c r="E14" s="146" t="s">
         <v>90</v>
       </c>
       <c r="F14" s="36">
@@ -16967,7 +17003,7 @@
       <c r="CE14" s="14"/>
       <c r="CF14" s="14"/>
     </row>
-    <row r="15" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:84" ht="16" x14ac:dyDescent="0.4">
       <c r="A15" s="36" t="s">
         <v>83</v>
       </c>
@@ -16978,8 +17014,8 @@
       <c r="D15" s="37">
         <v>9</v>
       </c>
-      <c r="E15" s="36" t="s">
-        <v>77</v>
+      <c r="E15" s="147" t="s">
+        <v>79</v>
       </c>
       <c r="F15" s="36">
         <v>10</v>
@@ -17024,8 +17060,8 @@
       <c r="D16" s="37">
         <v>7</v>
       </c>
-      <c r="E16" s="141" t="s">
-        <v>79</v>
+      <c r="E16" s="140" t="s">
+        <v>90</v>
       </c>
       <c r="F16" s="39">
         <v>3</v>
@@ -17591,7 +17627,7 @@
       <c r="D27" s="37">
         <v>6</v>
       </c>
-      <c r="E27" s="142" t="s">
+      <c r="E27" s="141" t="s">
         <v>536</v>
       </c>
       <c r="F27" s="40">
@@ -17638,7 +17674,7 @@
       <c r="D28" s="40">
         <v>4</v>
       </c>
-      <c r="E28" s="142" t="s">
+      <c r="E28" s="141" t="s">
         <v>536</v>
       </c>
       <c r="F28" s="39">
@@ -17737,7 +17773,7 @@
       <c r="D29" s="40">
         <v>4</v>
       </c>
-      <c r="E29" s="142" t="s">
+      <c r="E29" s="141" t="s">
         <v>90</v>
       </c>
       <c r="F29" s="39">
@@ -18116,7 +18152,7 @@
       <c r="B36" s="36"/>
       <c r="C36" s="139"/>
       <c r="D36" s="37"/>
-      <c r="E36" s="143" t="s">
+      <c r="E36" s="142" t="s">
         <v>536</v>
       </c>
       <c r="F36" s="39">
@@ -18138,7 +18174,7 @@
       <c r="D37" s="37">
         <v>10</v>
       </c>
-      <c r="E37" s="142" t="s">
+      <c r="E37" s="141" t="s">
         <v>90</v>
       </c>
       <c r="F37" s="39">
@@ -18424,7 +18460,7 @@
       <c r="D43" s="40">
         <v>5</v>
       </c>
-      <c r="E43" s="142" t="s">
+      <c r="E43" s="141" t="s">
         <v>92</v>
       </c>
       <c r="F43" s="39">
@@ -18516,7 +18552,7 @@
       <c r="D45" s="40">
         <v>5</v>
       </c>
-      <c r="E45" s="141" t="s">
+      <c r="E45" s="140" t="s">
         <v>537</v>
       </c>
       <c r="F45" s="39">
@@ -18661,7 +18697,7 @@
       <c r="D47" s="40">
         <v>5</v>
       </c>
-      <c r="E47" s="142" t="s">
+      <c r="E47" s="141" t="s">
         <v>90</v>
       </c>
       <c r="F47" s="39">
@@ -18950,10 +18986,10 @@
       <c r="G52" s="116"/>
     </row>
     <row r="53" spans="1:32" ht="16" x14ac:dyDescent="0.4">
-      <c r="A53" s="144" t="s">
+      <c r="A53" s="143" t="s">
         <v>267</v>
       </c>
-      <c r="B53" s="144"/>
+      <c r="B53" s="143"/>
       <c r="C53" s="41">
         <v>6000000141</v>
       </c>
@@ -18962,7 +18998,7 @@
         <v>90</v>
       </c>
       <c r="F53" s="75"/>
-      <c r="G53" s="145"/>
+      <c r="G53" s="144"/>
       <c r="H53" s="62"/>
       <c r="I53" s="62"/>
       <c r="J53" s="62"/>
@@ -21918,10 +21954,10 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="147" t="s">
+      <c r="A12" s="149" t="s">
         <v>132</v>
       </c>
-      <c r="B12" s="146">
+      <c r="B12" s="148">
         <v>6000000109</v>
       </c>
       <c r="D12" s="12" t="s">
@@ -21929,20 +21965,20 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="147"/>
-      <c r="B13" s="146"/>
+      <c r="A13" s="149"/>
+      <c r="B13" s="148"/>
       <c r="D13" s="21" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B14" s="148"/>
-      <c r="C14" s="149"/>
+      <c r="B14" s="150"/>
+      <c r="C14" s="151"/>
       <c r="D14" s="10"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B15" s="148"/>
-      <c r="C15" s="149"/>
+      <c r="B15" s="150"/>
+      <c r="C15" s="151"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -59507,7 +59543,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A3" s="155" t="s">
+      <c r="A3" s="157" t="s">
         <v>435</v>
       </c>
       <c r="B3" s="11" t="s">
@@ -59527,7 +59563,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A4" s="154"/>
+      <c r="A4" s="156"/>
       <c r="B4" s="67" t="s">
         <v>171</v>
       </c>
@@ -59543,7 +59579,7 @@
       <c r="F4" s="79"/>
     </row>
     <row r="5" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="151" t="s">
+      <c r="A5" s="153" t="s">
         <v>438</v>
       </c>
       <c r="B5" s="69" t="s">
@@ -59563,7 +59599,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A6" s="151"/>
+      <c r="A6" s="153"/>
       <c r="B6" s="69" t="s">
         <v>165</v>
       </c>
@@ -59579,7 +59615,7 @@
       <c r="F6" s="80"/>
     </row>
     <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A7" s="152"/>
+      <c r="A7" s="154"/>
       <c r="B7" s="69" t="s">
         <v>161</v>
       </c>
@@ -59595,7 +59631,7 @@
       <c r="F7" s="80"/>
     </row>
     <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A8" s="153" t="s">
+      <c r="A8" s="155" t="s">
         <v>441</v>
       </c>
       <c r="B8" s="11" t="s">
@@ -59615,7 +59651,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A9" s="154"/>
+      <c r="A9" s="156"/>
       <c r="B9" s="11" t="s">
         <v>179</v>
       </c>
@@ -59669,7 +59705,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A12" s="153" t="s">
+      <c r="A12" s="155" t="s">
         <v>446</v>
       </c>
       <c r="B12" s="11" t="s">
@@ -59687,7 +59723,7 @@
       <c r="F12" s="79"/>
     </row>
     <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A13" s="153"/>
+      <c r="A13" s="155"/>
       <c r="B13" s="11" t="s">
         <v>194</v>
       </c>
@@ -59703,7 +59739,7 @@
       <c r="F13" s="79"/>
     </row>
     <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A14" s="154"/>
+      <c r="A14" s="156"/>
       <c r="B14" s="11" t="s">
         <v>186</v>
       </c>
@@ -59833,7 +59869,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A21" s="153" t="s">
+      <c r="A21" s="155" t="s">
         <v>453</v>
       </c>
       <c r="B21" s="67" t="s">
@@ -59853,7 +59889,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A22" s="154"/>
+      <c r="A22" s="156"/>
       <c r="B22" s="11" t="s">
         <v>215</v>
       </c>
@@ -59869,7 +59905,7 @@
       <c r="F22" s="79"/>
     </row>
     <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A23" s="153" t="s">
+      <c r="A23" s="155" t="s">
         <v>454</v>
       </c>
       <c r="B23" s="11" t="s">
@@ -59889,7 +59925,7 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A24" s="153"/>
+      <c r="A24" s="155"/>
       <c r="B24" s="11" t="s">
         <v>219</v>
       </c>
@@ -59905,7 +59941,7 @@
       <c r="F24" s="79"/>
     </row>
     <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A25" s="154"/>
+      <c r="A25" s="156"/>
       <c r="B25" s="11" t="s">
         <v>221</v>
       </c>
@@ -59993,7 +60029,7 @@
       <c r="F29" s="79"/>
     </row>
     <row r="30" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A30" s="161" t="s">
+      <c r="A30" s="163" t="s">
         <v>459</v>
       </c>
       <c r="B30" s="108" t="s">
@@ -60011,7 +60047,7 @@
       <c r="F30" s="79"/>
     </row>
     <row r="31" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A31" s="161"/>
+      <c r="A31" s="163"/>
       <c r="B31" s="109" t="s">
         <v>409</v>
       </c>
@@ -60027,7 +60063,7 @@
       <c r="F31" s="79"/>
     </row>
     <row r="32" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A32" s="161"/>
+      <c r="A32" s="163"/>
       <c r="B32" s="109" t="s">
         <v>411</v>
       </c>
@@ -60079,7 +60115,7 @@
       <c r="F34" s="79"/>
     </row>
     <row r="35" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A35" s="153" t="s">
+      <c r="A35" s="155" t="s">
         <v>462</v>
       </c>
       <c r="B35" s="11" t="s">
@@ -60099,7 +60135,7 @@
       </c>
     </row>
     <row r="36" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A36" s="153"/>
+      <c r="A36" s="155"/>
       <c r="B36" s="68" t="s">
         <v>225</v>
       </c>
@@ -60117,7 +60153,7 @@
       </c>
     </row>
     <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A37" s="153"/>
+      <c r="A37" s="155"/>
       <c r="B37" s="68" t="s">
         <v>227</v>
       </c>
@@ -60135,7 +60171,7 @@
       </c>
     </row>
     <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A38" s="153"/>
+      <c r="A38" s="155"/>
       <c r="B38" s="67" t="s">
         <v>229</v>
       </c>
@@ -60153,7 +60189,7 @@
       </c>
     </row>
     <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A39" s="159"/>
+      <c r="A39" s="161"/>
       <c r="B39" s="11" t="s">
         <v>230</v>
       </c>
@@ -60271,7 +60307,7 @@
       </c>
     </row>
     <row r="45" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A45" s="161" t="s">
+      <c r="A45" s="163" t="s">
         <v>470</v>
       </c>
       <c r="B45" s="11" t="s">
@@ -60291,7 +60327,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A46" s="163"/>
+      <c r="A46" s="165"/>
       <c r="B46" s="11" t="s">
         <v>247</v>
       </c>
@@ -60309,7 +60345,7 @@
       </c>
     </row>
     <row r="47" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A47" s="153" t="s">
+      <c r="A47" s="155" t="s">
         <v>471</v>
       </c>
       <c r="B47" s="11" t="s">
@@ -60329,7 +60365,7 @@
       </c>
     </row>
     <row r="48" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A48" s="153"/>
+      <c r="A48" s="155"/>
       <c r="B48" s="11" t="s">
         <v>251</v>
       </c>
@@ -60387,7 +60423,7 @@
       </c>
     </row>
     <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A51" s="162" t="s">
+      <c r="A51" s="164" t="s">
         <v>475</v>
       </c>
       <c r="B51" s="22" t="s">
@@ -60403,7 +60439,7 @@
       <c r="F51" s="71"/>
     </row>
     <row r="52" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A52" s="162"/>
+      <c r="A52" s="164"/>
       <c r="B52" s="22" t="s">
         <v>130</v>
       </c>
@@ -60419,7 +60455,7 @@
       </c>
     </row>
     <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A53" s="162" t="s">
+      <c r="A53" s="164" t="s">
         <v>475</v>
       </c>
       <c r="B53" s="22" t="s">
@@ -60437,7 +60473,7 @@
       </c>
     </row>
     <row r="54" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A54" s="162"/>
+      <c r="A54" s="164"/>
       <c r="B54" s="22" t="s">
         <v>126</v>
       </c>
@@ -60453,7 +60489,7 @@
       </c>
     </row>
     <row r="55" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A55" s="153" t="s">
+      <c r="A55" s="155" t="s">
         <v>476</v>
       </c>
       <c r="B55" s="67" t="s">
@@ -60473,7 +60509,7 @@
       </c>
     </row>
     <row r="56" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A56" s="153"/>
+      <c r="A56" s="155"/>
       <c r="B56" s="11" t="s">
         <v>268</v>
       </c>
@@ -60491,7 +60527,7 @@
       </c>
     </row>
     <row r="57" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A57" s="154"/>
+      <c r="A57" s="156"/>
       <c r="B57" s="11" t="s">
         <v>269</v>
       </c>
@@ -60601,7 +60637,7 @@
       <c r="F62" s="70"/>
     </row>
     <row r="63" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A63" s="160" t="s">
+      <c r="A63" s="162" t="s">
         <v>482</v>
       </c>
       <c r="B63" s="75" t="s">
@@ -60619,7 +60655,7 @@
       <c r="F63" s="70"/>
     </row>
     <row r="64" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A64" s="160"/>
+      <c r="A64" s="162"/>
       <c r="B64" s="75" t="s">
         <v>401</v>
       </c>
@@ -60671,7 +60707,7 @@
       <c r="F66" s="70"/>
     </row>
     <row r="67" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A67" s="153" t="s">
+      <c r="A67" s="155" t="s">
         <v>485</v>
       </c>
       <c r="B67" s="11" t="s">
@@ -60691,7 +60727,7 @@
       </c>
     </row>
     <row r="68" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A68" s="153"/>
+      <c r="A68" s="155"/>
       <c r="B68" s="11" t="s">
         <v>276</v>
       </c>
@@ -60709,7 +60745,7 @@
       </c>
     </row>
     <row r="69" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A69" s="154"/>
+      <c r="A69" s="156"/>
       <c r="B69" s="11" t="s">
         <v>277</v>
       </c>
@@ -60747,7 +60783,7 @@
       </c>
     </row>
     <row r="71" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A71" s="153" t="s">
+      <c r="A71" s="155" t="s">
         <v>487</v>
       </c>
       <c r="B71" s="11" t="s">
@@ -60767,7 +60803,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A72" s="153"/>
+      <c r="A72" s="155"/>
       <c r="B72" s="11" t="s">
         <v>281</v>
       </c>
@@ -60823,7 +60859,7 @@
       </c>
     </row>
     <row r="75" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A75" s="153" t="s">
+      <c r="A75" s="155" t="s">
         <v>491</v>
       </c>
       <c r="B75" s="11" t="s">
@@ -60843,7 +60879,7 @@
       </c>
     </row>
     <row r="76" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A76" s="153"/>
+      <c r="A76" s="155"/>
       <c r="B76" s="11" t="s">
         <v>291</v>
       </c>
@@ -60881,7 +60917,7 @@
       </c>
     </row>
     <row r="78" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A78" s="153" t="s">
+      <c r="A78" s="155" t="s">
         <v>493</v>
       </c>
       <c r="B78" s="11" t="s">
@@ -60899,7 +60935,7 @@
       <c r="F78" s="70"/>
     </row>
     <row r="79" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A79" s="154"/>
+      <c r="A79" s="156"/>
       <c r="B79" s="11" t="s">
         <v>295</v>
       </c>
@@ -60937,7 +60973,7 @@
       </c>
     </row>
     <row r="81" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A81" s="153" t="s">
+      <c r="A81" s="155" t="s">
         <v>495</v>
       </c>
       <c r="B81" s="11" t="s">
@@ -60955,7 +60991,7 @@
       <c r="F81" s="70"/>
     </row>
     <row r="82" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A82" s="154"/>
+      <c r="A82" s="156"/>
       <c r="B82" s="11" t="s">
         <v>302</v>
       </c>
@@ -60973,7 +61009,7 @@
       </c>
     </row>
     <row r="83" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A83" s="166" t="s">
+      <c r="A83" s="168" t="s">
         <v>475</v>
       </c>
       <c r="B83" s="22" t="s">
@@ -60991,7 +61027,7 @@
       </c>
     </row>
     <row r="84" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A84" s="168"/>
+      <c r="A84" s="170"/>
       <c r="B84" s="22" t="s">
         <v>497</v>
       </c>
@@ -61065,7 +61101,7 @@
       </c>
     </row>
     <row r="88" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A88" s="166" t="s">
+      <c r="A88" s="168" t="s">
         <v>503</v>
       </c>
       <c r="B88" s="22" t="s">
@@ -61083,7 +61119,7 @@
       </c>
     </row>
     <row r="89" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A89" s="168"/>
+      <c r="A89" s="170"/>
       <c r="B89" s="22" t="s">
         <v>505</v>
       </c>
@@ -61099,7 +61135,7 @@
       </c>
     </row>
     <row r="90" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A90" s="153" t="s">
+      <c r="A90" s="155" t="s">
         <v>506</v>
       </c>
       <c r="B90" s="11" t="s">
@@ -61119,7 +61155,7 @@
       </c>
     </row>
     <row r="91" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A91" s="153"/>
+      <c r="A91" s="155"/>
       <c r="B91" s="68" t="s">
         <v>320</v>
       </c>
@@ -61137,7 +61173,7 @@
       </c>
     </row>
     <row r="92" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A92" s="153"/>
+      <c r="A92" s="155"/>
       <c r="B92" s="68" t="s">
         <v>320</v>
       </c>
@@ -61153,7 +61189,7 @@
       <c r="F92" s="70"/>
     </row>
     <row r="93" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A93" s="154"/>
+      <c r="A93" s="156"/>
       <c r="B93" s="67" t="s">
         <v>321</v>
       </c>
@@ -61171,7 +61207,7 @@
       </c>
     </row>
     <row r="94" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A94" s="153" t="s">
+      <c r="A94" s="155" t="s">
         <v>507</v>
       </c>
       <c r="B94" s="11" t="s">
@@ -61191,7 +61227,7 @@
       </c>
     </row>
     <row r="95" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A95" s="153"/>
+      <c r="A95" s="155"/>
       <c r="B95" s="11" t="s">
         <v>328</v>
       </c>
@@ -61209,7 +61245,7 @@
       </c>
     </row>
     <row r="96" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A96" s="159"/>
+      <c r="A96" s="161"/>
       <c r="B96" s="67" t="s">
         <v>331</v>
       </c>
@@ -61247,7 +61283,7 @@
       </c>
     </row>
     <row r="98" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A98" s="164" t="s">
+      <c r="A98" s="166" t="s">
         <v>509</v>
       </c>
       <c r="B98" s="67" t="s">
@@ -61267,7 +61303,7 @@
       </c>
     </row>
     <row r="99" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A99" s="164"/>
+      <c r="A99" s="166"/>
       <c r="B99" s="11" t="s">
         <v>343</v>
       </c>
@@ -61285,7 +61321,7 @@
       </c>
     </row>
     <row r="100" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A100" s="165"/>
+      <c r="A100" s="167"/>
       <c r="B100" s="11" t="s">
         <v>341</v>
       </c>
@@ -61323,7 +61359,7 @@
       </c>
     </row>
     <row r="102" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A102" s="153" t="s">
+      <c r="A102" s="155" t="s">
         <v>511</v>
       </c>
       <c r="B102" s="11" t="s">
@@ -61343,7 +61379,7 @@
       </c>
     </row>
     <row r="103" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A103" s="153"/>
+      <c r="A103" s="155"/>
       <c r="B103" s="11" t="s">
         <v>347</v>
       </c>
@@ -61361,7 +61397,7 @@
       </c>
     </row>
     <row r="104" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A104" s="159"/>
+      <c r="A104" s="161"/>
       <c r="B104" s="11" t="s">
         <v>349</v>
       </c>
@@ -61379,7 +61415,7 @@
       </c>
     </row>
     <row r="105" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A105" s="166" t="s">
+      <c r="A105" s="168" t="s">
         <v>514</v>
       </c>
       <c r="B105" s="22" t="s">
@@ -61397,7 +61433,7 @@
       </c>
     </row>
     <row r="106" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A106" s="166"/>
+      <c r="A106" s="168"/>
       <c r="B106" s="22" t="s">
         <v>122</v>
       </c>
@@ -61413,7 +61449,7 @@
       </c>
     </row>
     <row r="107" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A107" s="166"/>
+      <c r="A107" s="168"/>
       <c r="B107" s="22" t="s">
         <v>74</v>
       </c>
@@ -61429,7 +61465,7 @@
       </c>
     </row>
     <row r="108" spans="1:6" ht="16" x14ac:dyDescent="0.4">
-      <c r="A108" s="167"/>
+      <c r="A108" s="169"/>
       <c r="B108" s="22" t="s">
         <v>517</v>
       </c>
@@ -61731,7 +61767,7 @@
       </c>
     </row>
     <row r="124" spans="1:7" ht="16" x14ac:dyDescent="0.4">
-      <c r="A124" s="156" t="s">
+      <c r="A124" s="158" t="s">
         <v>533</v>
       </c>
       <c r="B124" s="119" t="s">
@@ -61754,7 +61790,7 @@
       </c>
     </row>
     <row r="125" spans="1:7" ht="16" x14ac:dyDescent="0.4">
-      <c r="A125" s="157"/>
+      <c r="A125" s="159"/>
       <c r="B125" s="119" t="s">
         <v>424</v>
       </c>
@@ -61775,7 +61811,7 @@
       </c>
     </row>
     <row r="126" spans="1:7" ht="16" x14ac:dyDescent="0.4">
-      <c r="A126" s="158"/>
+      <c r="A126" s="160"/>
       <c r="B126" s="119" t="s">
         <v>426</v>
       </c>
@@ -61823,7 +61859,7 @@
       <c r="F128" s="62"/>
     </row>
     <row r="129" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A129" s="150"/>
+      <c r="A129" s="152"/>
       <c r="B129" s="121"/>
       <c r="C129" s="62"/>
       <c r="D129" s="62"/>
@@ -61831,7 +61867,7 @@
       <c r="F129" s="62"/>
     </row>
     <row r="130" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A130" s="150"/>
+      <c r="A130" s="152"/>
       <c r="B130" s="121"/>
       <c r="C130" s="62"/>
       <c r="D130" s="62"/>

</xml_diff>